<commit_message>
Configure queue, credential asset and ACME URL asset in Config.xlsx
Set OrchestratorQueueName and logF_BusinessProcessName to
ACME_ClientSecurityHash, add ACME_CredentialAssetName to Settings and
the ACME_URL row to Assets. Retries are left to the queue.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="49">
   <si>
     <t>Name</t>
   </si>
@@ -87,7 +87,7 @@
     <t>logF_BusinessProcessName</t>
   </si>
   <si>
-    <t>Framework</t>
+    <t>ACME_CredentialAssetName</t>
   </si>
   <si>
     <t>Orchestrator queue Name. The value must match with the queue name defined on Orchestrator.</t>
@@ -102,7 +102,7 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>Must be 0 if working with Orchestrator queues. If &gt; 0, the robot will retry the same transaction which failed with a system exception. Must be an integer value.</t>
+    <t>Retries handled by Orchestrator queue auto-retry</t>
   </si>
   <si>
     <t>Static part of logging message. Processed Transaction succesful.</t>
@@ -159,7 +159,19 @@
     <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
   </si>
   <si>
-    <t>ProcessABCQueue</t>
+    <t>ACME_ClientSecurityHash</t>
+  </si>
+  <si>
+    <t>ACME_Credential</t>
+  </si>
+  <si>
+    <t>Name of the Orchestrator credential asset for ACME login</t>
+  </si>
+  <si>
+    <t>ACME_URL</t>
+  </si>
+  <si>
+    <t>ACME System 1 URL from Orchestrator text asset</t>
   </si>
 </sst>
 </file>
@@ -604,13 +616,23 @@
         <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
@@ -2815,7 +2837,17 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="2" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" t="s">
+        <v>48</v>
+      </c>
+    </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="5" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Open, close and kill applications from the framework
InitAllApplications logs in to ACME. CloseAllApplications closes both
sites and now receives Config, as does KillAllProcesses, which kills
Chrome only when KillChromeOnRecovery is TRUE. Add the related Config
settings. ProcessTestCase builds its queue item from an argument and
no longer takes one from the queue.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="67">
   <si>
     <t>Name</t>
   </si>
@@ -172,6 +172,60 @@
   </si>
   <si>
     <t>ACME System 1 URL from Orchestrator text asset</t>
+  </si>
+  <si>
+    <t>SHA1_URL</t>
+  </si>
+  <si>
+    <t>http://www.sha1-online.com/</t>
+  </si>
+  <si>
+    <t>Address of the SHA1 Online hash generator</t>
+  </si>
+  <si>
+    <t>SHA1_Algorithm</t>
+  </si>
+  <si>
+    <t>sha-1</t>
+  </si>
+  <si>
+    <t>Item to select in the hash algorithm dropdown of SHA1 Online</t>
+  </si>
+  <si>
+    <t>ACME_WorkItemType</t>
+  </si>
+  <si>
+    <t>WI5</t>
+  </si>
+  <si>
+    <t>Work item type this process handles; queue items of any other type are rejected as business exceptions</t>
+  </si>
+  <si>
+    <t>ACME_CompletedStatus</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Status set on a work item once its hash comment is added</t>
+  </si>
+  <si>
+    <t>ACME_UpdateSuccessText</t>
+  </si>
+  <si>
+    <t>Work Item was updated accordingly</t>
+  </si>
+  <si>
+    <t>Text of the browser alert ACME shows after a successful work item update</t>
+  </si>
+  <si>
+    <t>KillChromeOnRecovery</t>
+  </si>
+  <si>
+    <t>FALSE</t>
+  </si>
+  <si>
+    <t>TRUE to force-kill chrome.exe when applications cannot be closed. Keep FALSE on a machine where a person also uses Chrome</t>
   </si>
 </sst>
 </file>
@@ -633,12 +687,72 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A12" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="15" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Send exception emails over SMTP
Add SendExceptionEmail and call it in three places: a rejected ACME
login (PDD text, then the run ends), a system exception on a
transaction (with the screenshot), and a run stopped by a system
exception. The SMTP account comes from a credential asset; recipient,
server and port come from Config. With recipient or server empty the
message is logged instead of sent, and a send failure never replaces
the original exception.

Adds the UiPath.Mail.Activities dependency.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="80">
   <si>
     <t>Name</t>
   </si>
@@ -226,6 +226,45 @@
   </si>
   <si>
     <t>TRUE to force-kill chrome.exe when applications cannot be closed. Keep FALSE on a machine where a person also uses Chrome</t>
+  </si>
+  <si>
+    <t>ExceptionEmail_To</t>
+  </si>
+  <si>
+    <t>Recipient of exception emails (several addresses separated by semicolons). Leave empty to log the message instead of sending it</t>
+  </si>
+  <si>
+    <t>ExceptionEmail_LoginFailedBody</t>
+  </si>
+  <si>
+    <t>Hello, The username or the email is incorrect. Please check and restart Thank you</t>
+  </si>
+  <si>
+    <t>Body of the email sent when ACME rejects the login (text from the PDD)</t>
+  </si>
+  <si>
+    <t>SMTP_Server</t>
+  </si>
+  <si>
+    <t>SMTP server used to send exception emails, for example smtp.gmail.com. Leave empty to log the message instead of sending it</t>
+  </si>
+  <si>
+    <t>SMTP_Port</t>
+  </si>
+  <si>
+    <t>587</t>
+  </si>
+  <si>
+    <t>SMTP port (587 for STARTTLS, 465 for SSL)</t>
+  </si>
+  <si>
+    <t>SMTP_CredentialAssetName</t>
+  </si>
+  <si>
+    <t>SMTP_Credential</t>
+  </si>
+  <si>
+    <t>Name of the Orchestrator credential asset holding the sending mailbox address and its password</t>
   </si>
 </sst>
 </file>
@@ -753,11 +792,55 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" ht="14.25" customHeight="1"/>
+    <row r="13" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A13" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A16" t="s">
+        <v>74</v>
+      </c>
+      <c r="B16" t="s">
+        <v>75</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" ht="14.25" customHeight="1">
+      <c r="A17" t="s">
+        <v>77</v>
+      </c>
+      <c r="B17" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
     <row r="18" ht="14.25" customHeight="1"/>
     <row r="19" ht="14.25" customHeight="1"/>
     <row r="20" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Set the Orchestrator folder and SMTP server in Config; untrack local tooling files
Config: OrchestratorQueueFolder = ACME_Portfolio, SMTP_Server = smtp.gmail.com.
ExceptionEmail_To stays empty; fill it locally to switch exception emails on.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uipath-my.sharepoint.com/personal/alexandra_veizu_uipath_com/Documents/Documents/Projects/REFrameworkNET5/StudioTemplates/REFramework/contentFiles/any/any/pt2/VisualBasic/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UiPath\ACME_Performer\ACME_ClientHash_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{00D541BD-CB78-4D75-8532-9AD73E8C785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8C54E24-BA5C-4BF9-8DAB-2778512EC11B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ADB8CDB-FC6F-41FC-A966-B556B226A34F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="19416" windowHeight="11784" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="83">
   <si>
     <t>Name</t>
   </si>
@@ -162,116 +162,125 @@
     <t>ACME_ClientSecurityHash</t>
   </si>
   <si>
+    <t>Name of the Orchestrator credential asset for ACME login</t>
+  </si>
+  <si>
+    <t>ACME_URL</t>
+  </si>
+  <si>
+    <t>ACME System 1 URL from Orchestrator text asset</t>
+  </si>
+  <si>
+    <t>SHA1_URL</t>
+  </si>
+  <si>
+    <t>http://www.sha1-online.com/</t>
+  </si>
+  <si>
+    <t>Address of the SHA1 Online hash generator</t>
+  </si>
+  <si>
+    <t>SHA1_Algorithm</t>
+  </si>
+  <si>
+    <t>sha-1</t>
+  </si>
+  <si>
+    <t>Item to select in the hash algorithm dropdown of SHA1 Online</t>
+  </si>
+  <si>
+    <t>ACME_WorkItemType</t>
+  </si>
+  <si>
+    <t>WI5</t>
+  </si>
+  <si>
+    <t>Work item type this process handles; queue items of any other type are rejected as business exceptions</t>
+  </si>
+  <si>
+    <t>ACME_CompletedStatus</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Status set on a work item once its hash comment is added</t>
+  </si>
+  <si>
+    <t>ACME_UpdateSuccessText</t>
+  </si>
+  <si>
+    <t>Work Item was updated accordingly</t>
+  </si>
+  <si>
+    <t>Text of the browser alert ACME shows after a successful work item update</t>
+  </si>
+  <si>
+    <t>KillChromeOnRecovery</t>
+  </si>
+  <si>
+    <t>FALSE</t>
+  </si>
+  <si>
+    <t>TRUE to force-kill chrome.exe when applications cannot be closed. Keep FALSE on a machine where a person also uses Chrome</t>
+  </si>
+  <si>
+    <t>ExceptionEmail_To</t>
+  </si>
+  <si>
+    <t>Recipient of exception emails (several addresses separated by semicolons). Leave empty to log the message instead of sending it</t>
+  </si>
+  <si>
+    <t>ExceptionEmail_LoginFailedBody</t>
+  </si>
+  <si>
+    <t>Body of the email sent when ACME rejects the login (text from the PDD)</t>
+  </si>
+  <si>
+    <t>SMTP_Server</t>
+  </si>
+  <si>
+    <t>SMTP server used to send exception emails, for example smtp.gmail.com. Leave empty to log the message instead of sending it</t>
+  </si>
+  <si>
+    <t>SMTP_Port</t>
+  </si>
+  <si>
+    <t>587</t>
+  </si>
+  <si>
+    <t>SMTP port (587 for STARTTLS, 465 for SSL)</t>
+  </si>
+  <si>
+    <t>SMTP_CredentialAssetName</t>
+  </si>
+  <si>
+    <t>SMTP_Credential</t>
+  </si>
+  <si>
+    <t>Name of the Orchestrator credential asset holding the sending mailbox address and its password</t>
+  </si>
+  <si>
+    <t>ACME_Portfolio</t>
+  </si>
+  <si>
+    <t>smtp.gmail.com</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Hello, The password or the email is incorrect. Please check and restart Thank you</t>
+  </si>
+  <si>
     <t>ACME_Credential</t>
-  </si>
-  <si>
-    <t>Name of the Orchestrator credential asset for ACME login</t>
-  </si>
-  <si>
-    <t>ACME_URL</t>
-  </si>
-  <si>
-    <t>ACME System 1 URL from Orchestrator text asset</t>
-  </si>
-  <si>
-    <t>SHA1_URL</t>
-  </si>
-  <si>
-    <t>http://www.sha1-online.com/</t>
-  </si>
-  <si>
-    <t>Address of the SHA1 Online hash generator</t>
-  </si>
-  <si>
-    <t>SHA1_Algorithm</t>
-  </si>
-  <si>
-    <t>sha-1</t>
-  </si>
-  <si>
-    <t>Item to select in the hash algorithm dropdown of SHA1 Online</t>
-  </si>
-  <si>
-    <t>ACME_WorkItemType</t>
-  </si>
-  <si>
-    <t>WI5</t>
-  </si>
-  <si>
-    <t>Work item type this process handles; queue items of any other type are rejected as business exceptions</t>
-  </si>
-  <si>
-    <t>ACME_CompletedStatus</t>
-  </si>
-  <si>
-    <t>Completed</t>
-  </si>
-  <si>
-    <t>Status set on a work item once its hash comment is added</t>
-  </si>
-  <si>
-    <t>ACME_UpdateSuccessText</t>
-  </si>
-  <si>
-    <t>Work Item was updated accordingly</t>
-  </si>
-  <si>
-    <t>Text of the browser alert ACME shows after a successful work item update</t>
-  </si>
-  <si>
-    <t>KillChromeOnRecovery</t>
-  </si>
-  <si>
-    <t>FALSE</t>
-  </si>
-  <si>
-    <t>TRUE to force-kill chrome.exe when applications cannot be closed. Keep FALSE on a machine where a person also uses Chrome</t>
-  </si>
-  <si>
-    <t>ExceptionEmail_To</t>
-  </si>
-  <si>
-    <t>Recipient of exception emails (several addresses separated by semicolons). Leave empty to log the message instead of sending it</t>
-  </si>
-  <si>
-    <t>ExceptionEmail_LoginFailedBody</t>
-  </si>
-  <si>
-    <t>Hello, The username or the email is incorrect. Please check and restart Thank you</t>
-  </si>
-  <si>
-    <t>Body of the email sent when ACME rejects the login (text from the PDD)</t>
-  </si>
-  <si>
-    <t>SMTP_Server</t>
-  </si>
-  <si>
-    <t>SMTP server used to send exception emails, for example smtp.gmail.com. Leave empty to log the message instead of sending it</t>
-  </si>
-  <si>
-    <t>SMTP_Port</t>
-  </si>
-  <si>
-    <t>587</t>
-  </si>
-  <si>
-    <t>SMTP port (587 for STARTTLS, 465 for SSL)</t>
-  </si>
-  <si>
-    <t>SMTP_CredentialAssetName</t>
-  </si>
-  <si>
-    <t>SMTP_Credential</t>
-  </si>
-  <si>
-    <t>Name of the Orchestrator credential asset holding the sending mailbox address and its password</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -295,6 +304,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -313,10 +328,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -326,8 +342,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -698,7 +716,9 @@
       <c r="A3" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="2"/>
+      <c r="B3" s="2" t="s">
+        <v>78</v>
+      </c>
       <c r="C3" s="4" t="s">
         <v>32</v>
       </c>
@@ -720,142 +740,145 @@
         <v>21</v>
       </c>
       <c r="B6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" t="s">
         <v>52</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" s="4" t="s">
         <v>53</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" t="s">
         <v>55</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" s="4" t="s">
         <v>56</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" t="s">
         <v>58</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" s="4" t="s">
         <v>59</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" t="s">
         <v>61</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" s="4" t="s">
         <v>62</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" t="s">
         <v>64</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" t="s">
         <v>49</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" s="4" t="s">
         <v>50</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>67</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
+        <v>68</v>
+      </c>
+      <c r="B14" t="s">
+        <v>81</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="B14" t="s">
-        <v>70</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>72</v>
+        <v>70</v>
+      </c>
+      <c r="B15" t="s">
+        <v>79</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
+        <v>72</v>
+      </c>
+      <c r="B16" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B16" t="s">
+    </row>
+    <row r="17" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A17" t="s">
         <v>75</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="B17" t="s">
         <v>76</v>
       </c>
+      <c r="C17" s="4" t="s">
+        <v>77</v>
+      </c>
     </row>
-    <row r="17" ht="14.25" customHeight="1">
-      <c r="A17" t="s">
-        <v>77</v>
-      </c>
-      <c r="B17" t="s">
-        <v>78</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="18" ht="14.25" customHeight="1"/>
-    <row r="19" ht="14.25" customHeight="1"/>
-    <row r="20" ht="14.25" customHeight="1"/>
-    <row r="21" ht="14.25" customHeight="1"/>
-    <row r="22" ht="14.25" customHeight="1"/>
-    <row r="23" ht="14.25" customHeight="1"/>
-    <row r="24" ht="14.25" customHeight="1"/>
-    <row r="25" ht="14.25" customHeight="1"/>
-    <row r="26" ht="14.25" customHeight="1"/>
-    <row r="27" ht="14.25" customHeight="1"/>
-    <row r="28" ht="14.25" customHeight="1"/>
-    <row r="29" ht="14.25" customHeight="1"/>
-    <row r="30" ht="14.25" customHeight="1"/>
-    <row r="31" ht="14.25" customHeight="1"/>
-    <row r="32" ht="14.25" customHeight="1"/>
+    <row r="18" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="19" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="20" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="21" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="22" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="23" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="24" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="25" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="26" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="27" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="28" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="29" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="30" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="31" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="32" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="33" ht="14.25" customHeight="1"/>
     <row r="34" ht="14.25" customHeight="1"/>
     <row r="35" ht="14.25" customHeight="1"/>
@@ -1825,7 +1848,7 @@
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1874,7 +1897,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="28.8">
+    <row r="2" spans="1:26" ht="14.4">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -3036,13 +3059,16 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" t="s">
         <v>47</v>
-      </c>
-      <c r="B2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>